<commit_message>
"created a frontend ui dashboard, customers tab and there view."
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>a790cccb-82d4-4c70-96d2-9e980ae785e6</t>
+          <t>9e3e2dff-edba-4e00-9fd0-fda6e268cdab</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>QBE-820</t>
+          <t>QBE-751</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Industrial Dolore 39mm</t>
+          <t>Industrial Dolore 34mm</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -517,17 +517,17 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>960.9</v>
+        <v>3074.62</v>
       </c>
       <c r="H2" t="n">
-        <v>1196.37</v>
+        <v>3806.63</v>
       </c>
       <c r="I2" t="n">
-        <v>73</v>
+        <v>694</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Monsoon</t>
         </is>
       </c>
       <c r="K2" t="b">
@@ -537,7 +537,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ead119ad-8d0c-40e9-8349-08693917a240</t>
+          <t>8682fb4a-79b8-40f6-96b3-0a4ef96ceaec</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -547,36 +547,36 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IOI-179</t>
+          <t>IOI-416</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Industrial Mollitia 50mm</t>
+          <t>Industrial Mollitia 66mm</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>307.28</v>
+        <v>4526.68</v>
       </c>
       <c r="H3" t="n">
-        <v>354.81</v>
+        <v>5937.13</v>
       </c>
       <c r="I3" t="n">
-        <v>587</v>
+        <v>749</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Monsoon</t>
         </is>
       </c>
       <c r="K3" t="b">
@@ -586,7 +586,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>06831554-322e-420f-b9ee-4e8bc6a8968f</t>
+          <t>d62de34f-03d4-4679-b638-69abe3a8db63</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -596,12 +596,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>YZI-121</t>
+          <t>YZI-279</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Industrial Impedit 51mm</t>
+          <t>Industrial Impedit 35mm</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -611,17 +611,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2146.7</v>
+        <v>1546.04</v>
       </c>
       <c r="H4" t="n">
-        <v>2530.52</v>
+        <v>2066.85</v>
       </c>
       <c r="I4" t="n">
-        <v>851</v>
+        <v>543</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fdeca01b-d477-4c91-8288-3f0667fb2a03</t>
+          <t>8623f40c-3210-4857-aafb-d7766f0784ff</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -645,17 +645,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>OJT-703</t>
+          <t>OJT-593</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Industrial Veritatis 61mm</t>
+          <t>Industrial Veritatis 47mm</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -664,19 +664,15 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4237.97</v>
+        <v>1359.15</v>
       </c>
       <c r="H5" t="n">
-        <v>5131.46</v>
+        <v>1843.24</v>
       </c>
       <c r="I5" t="n">
-        <v>405</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Summer</t>
-        </is>
-      </c>
+        <v>479</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="b">
         <v>0</v>
       </c>
@@ -684,7 +680,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d040feee-47dc-4805-b73b-c7bc41c12878</t>
+          <t>be325d35-8cdf-42f3-af42-743bc982fd37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -694,46 +690,46 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>YUP-178</t>
+          <t>YUP-841</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Industrial Minima 75mm</t>
+          <t>Industrial Minima 96mm</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fittings</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1185.7</v>
+        <v>4835.85</v>
       </c>
       <c r="H6" t="n">
-        <v>1594.51</v>
+        <v>6601.11</v>
       </c>
       <c r="I6" t="n">
-        <v>927</v>
+        <v>92</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Summer</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>b0c08a25-ec0c-49fa-8e09-4bc53cc92036</t>
+          <t>7155a35e-d8bc-439d-8ff0-bc996d46be76</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -743,36 +739,36 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AJJ-251</t>
+          <t>AJJ-788</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Industrial Dicta 40mm</t>
+          <t>Industrial Dicta 96mm</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fittings</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Meters</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>4795.29</v>
+        <v>2729.2</v>
       </c>
       <c r="H7" t="n">
-        <v>6288.36</v>
+        <v>3448.88</v>
       </c>
       <c r="I7" t="n">
-        <v>262</v>
+        <v>842</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Summer</t>
         </is>
       </c>
       <c r="K7" t="b">
@@ -782,7 +778,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>b7306db2-63de-45c6-b1f3-7bf9cb7e43ab</t>
+          <t>6228b740-5af7-464c-9427-2e5650d0229b</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -792,38 +788,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HCA-177</t>
+          <t>HCA-674</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Industrial Rem 32mm</t>
+          <t>Industrial Rem 51mm</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>849.0599999999999</v>
+        <v>1245.73</v>
       </c>
       <c r="H8" t="n">
-        <v>1137.56</v>
+        <v>1440.38</v>
       </c>
       <c r="I8" t="n">
-        <v>772</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Winter</t>
-        </is>
-      </c>
+        <v>663</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="b">
         <v>0</v>
       </c>
@@ -831,7 +823,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6d140a61-29c3-4032-9fdb-7f84fa9467c2</t>
+          <t>564a9136-aebd-4f0d-a467-33a48ffa93e7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -841,17 +833,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MZI-739</t>
+          <t>MZI-764</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Industrial Quo 51mm</t>
+          <t>Industrial Quo 62mm</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -860,13 +852,13 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>4422.04</v>
+        <v>2374.91</v>
       </c>
       <c r="H9" t="n">
-        <v>5796.18</v>
+        <v>3147.4</v>
       </c>
       <c r="I9" t="n">
-        <v>450</v>
+        <v>46</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="b">
@@ -876,7 +868,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0d4f12cc-a18e-4222-a03e-cd5b5cf6b577</t>
+          <t>55a2b589-8f30-40f8-a95d-5a455ff32c5a</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -886,32 +878,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FTN-705</t>
+          <t>FTN-650</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Industrial Laborum 17mm</t>
+          <t>Industrial Laborum 27mm</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Meters</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3193.79</v>
+        <v>2513.86</v>
       </c>
       <c r="H10" t="n">
-        <v>4308.69</v>
+        <v>2952.02</v>
       </c>
       <c r="I10" t="n">
-        <v>317</v>
+        <v>379</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -925,7 +917,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8ba01fde-8041-42ea-b761-0a889b2df402</t>
+          <t>5b36a7f3-fcaf-47dd-a9fb-9378d2f90164</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -935,17 +927,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NAP-178</t>
+          <t>NAP-770</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Industrial Quam 92mm</t>
+          <t>Industrial Quam 22mm</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fittings</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -954,23 +946,27 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>378.76</v>
+        <v>3660.34</v>
       </c>
       <c r="H11" t="n">
-        <v>514.33</v>
+        <v>5019.62</v>
       </c>
       <c r="I11" t="n">
-        <v>473</v>
-      </c>
-      <c r="J11" t="inlineStr"/>
+        <v>961</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Summer</t>
+        </is>
+      </c>
       <c r="K11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cf291a6c-3b12-451e-837d-b7e5555e6590</t>
+          <t>5de3e2ce-6136-402a-afb1-adbe07312074</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -980,34 +976,38 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JKL-429</t>
+          <t>JKL-341</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Industrial Est 87mm</t>
+          <t>Industrial Est 56mm</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>4068.1</v>
+        <v>1915.6</v>
       </c>
       <c r="H12" t="n">
-        <v>5341.25</v>
+        <v>2415.28</v>
       </c>
       <c r="I12" t="n">
-        <v>980</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>557</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Summer</t>
+        </is>
+      </c>
       <c r="K12" t="b">
         <v>0</v>
       </c>
@@ -1015,7 +1015,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>202b0978-03f7-4d03-a4d5-b9a8b4a7736f</t>
+          <t>ea5cbb32-2237-4bf2-a204-bc0aef8f9fc2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1025,17 +1025,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NQM-831</t>
+          <t>NQM-968</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Industrial Cum 20mm</t>
+          <t>Industrial Cum 68mm</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1044,19 +1044,15 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>4073.74</v>
+        <v>1451.82</v>
       </c>
       <c r="H13" t="n">
-        <v>5537.62</v>
+        <v>2021.01</v>
       </c>
       <c r="I13" t="n">
-        <v>40</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Monsoon</t>
-        </is>
-      </c>
+        <v>657</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="b">
         <v>0</v>
       </c>
@@ -1064,7 +1060,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>edeb3e6e-d391-4fde-b482-35923a3956c0</t>
+          <t>c571d368-d220-4a3a-ac44-79585b3eb6f9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1074,36 +1070,36 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LQZ-724</t>
+          <t>LQZ-905</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Industrial Reiciendis 30mm</t>
+          <t>Industrial Reiciendis 82mm</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pipes</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Box</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>4955.83</v>
+        <v>1734.19</v>
       </c>
       <c r="H14" t="n">
-        <v>6348.5</v>
+        <v>2423.02</v>
       </c>
       <c r="I14" t="n">
-        <v>939</v>
+        <v>849</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Summer</t>
+          <t>Monsoon</t>
         </is>
       </c>
       <c r="K14" t="b">
@@ -1113,7 +1109,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>a1808d5e-2b25-498a-921d-5923b3e205be</t>
+          <t>b5819597-555f-4453-838b-8815df269f35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1123,17 +1119,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DWJ-153</t>
+          <t>DWJ-892</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Industrial Officiis 90mm</t>
+          <t>Industrial Officiis 28mm</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1142,15 +1138,19 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>3894.88</v>
+        <v>4083.96</v>
       </c>
       <c r="H15" t="n">
-        <v>5140.17</v>
+        <v>4934.44</v>
       </c>
       <c r="I15" t="n">
-        <v>337</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>283</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Monsoon</t>
+        </is>
+      </c>
       <c r="K15" t="b">
         <v>0</v>
       </c>
@@ -1158,7 +1158,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3db97d61-d3e6-4f3d-a6e4-bfdc1c78509b</t>
+          <t>c92281f3-88ed-4239-b105-e015e87c1eb5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PJE-972</t>
+          <t>PJE-212</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1187,15 +1187,19 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1994.16</v>
+        <v>2747.06</v>
       </c>
       <c r="H16" t="n">
-        <v>2418.91</v>
+        <v>3707.51</v>
       </c>
       <c r="I16" t="n">
-        <v>341</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Summer</t>
+        </is>
+      </c>
       <c r="K16" t="b">
         <v>0</v>
       </c>
@@ -1203,7 +1207,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>55e0fb72-dc35-43d0-a3a6-23fda72e18ca</t>
+          <t>3912843c-002d-4bb3-a918-04e627e1ef9b</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1213,17 +1217,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>QEQ-771</t>
+          <t>QEQ-278</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Industrial Consequuntur 99mm</t>
+          <t>Industrial Consequuntur 43mm</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1232,15 +1236,19 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>793</v>
+        <v>1265.86</v>
       </c>
       <c r="H17" t="n">
-        <v>981.3</v>
+        <v>1558.2</v>
       </c>
       <c r="I17" t="n">
-        <v>609</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
+        <v>759</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Winter</t>
+        </is>
+      </c>
       <c r="K17" t="b">
         <v>0</v>
       </c>
@@ -1248,7 +1256,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2fcf896f-bcb0-4ca3-826c-da60bc0419b9</t>
+          <t>09b0c4d1-bde3-4feb-ad36-2d85e9b09d24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1258,12 +1266,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MUL-932</t>
+          <t>MUL-896</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Industrial Placeat 26mm</t>
+          <t>Industrial Placeat 56mm</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1277,17 +1285,17 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1945.73</v>
+        <v>3753.76</v>
       </c>
       <c r="H18" t="n">
-        <v>2622.68</v>
+        <v>4763.75</v>
       </c>
       <c r="I18" t="n">
-        <v>661</v>
+        <v>462</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Monsoon</t>
         </is>
       </c>
       <c r="K18" t="b">
@@ -1297,7 +1305,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>81d858ed-96f9-4144-8a86-a5b419dd74c0</t>
+          <t>cf390282-c34b-4d69-86a6-15afede8f222</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1307,38 +1315,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>VWI-319</t>
+          <t>VWI-987</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Industrial Velit 53mm</t>
+          <t>Industrial Velit 94mm</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>189.33</v>
+        <v>312.49</v>
       </c>
       <c r="H19" t="n">
-        <v>232.35</v>
+        <v>420.55</v>
       </c>
       <c r="I19" t="n">
-        <v>231</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Monsoon</t>
-        </is>
-      </c>
+        <v>469</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="b">
         <v>0</v>
       </c>
@@ -1346,7 +1350,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>d223c82c-137d-4c90-8d33-64c3b77bebba</t>
+          <t>4934f762-fedf-4321-b775-7f184a8ea0c4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1356,38 +1360,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PPG-619</t>
+          <t>PPG-802</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Industrial Id 79mm</t>
+          <t>Industrial Id 23mm</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Meters</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1549.38</v>
+        <v>2447.01</v>
       </c>
       <c r="H20" t="n">
-        <v>2087.06</v>
+        <v>3059.75</v>
       </c>
       <c r="I20" t="n">
-        <v>677</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Summer</t>
-        </is>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="b">
         <v>0</v>
       </c>
@@ -1395,7 +1395,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>8c4a649a-1ddd-4102-8a8f-f14908ec1610</t>
+          <t>39bfaa70-d6b0-4753-9188-1d94a54b1299</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1405,46 +1405,46 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NEM-257</t>
+          <t>NEM-739</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Industrial Ipsum 30mm</t>
+          <t>Industrial Ipsum 91mm</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>3128.35</v>
+        <v>826.84</v>
       </c>
       <c r="H21" t="n">
-        <v>4064.7</v>
+        <v>976.95</v>
       </c>
       <c r="I21" t="n">
-        <v>738</v>
+        <v>390</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Summer</t>
         </is>
       </c>
       <c r="K21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7294ca2b-f2c7-4436-b9b0-698070e56602</t>
+          <t>f2970769-9ab5-49d8-b0e8-ceea2680e13e</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1454,36 +1454,36 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FCV-554</t>
+          <t>FCV-818</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Industrial Sint 88mm</t>
+          <t>Industrial Sint 24mm</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1885.07</v>
+        <v>3066.59</v>
       </c>
       <c r="H22" t="n">
-        <v>2506.95</v>
+        <v>3602.61</v>
       </c>
       <c r="I22" t="n">
-        <v>239</v>
+        <v>440</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K22" t="b">
@@ -1493,7 +1493,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>45e750d8-3fd6-48e5-94c6-3a4e5c288a37</t>
+          <t>f3970cb0-a168-4b34-9069-096c1901f713</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1503,32 +1503,32 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>QTS-955</t>
+          <t>QTS-508</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Industrial Reprehenderit 34mm</t>
+          <t>Industrial Reprehenderit 63mm</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>4062.26</v>
+        <v>2127.69</v>
       </c>
       <c r="H23" t="n">
-        <v>5147.91</v>
+        <v>2886.97</v>
       </c>
       <c r="I23" t="n">
-        <v>472</v>
+        <v>437</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1613725e-ceb7-46bb-ae49-792e9a7c038f</t>
+          <t>d7098c25-3ec8-4753-b1f5-02c60d4ae30c</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1552,36 +1552,36 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JKK-265</t>
+          <t>JKK-585</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Industrial Maiores 35mm</t>
+          <t>Industrial Maiores 18mm</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Box</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2564.24</v>
+        <v>1934.08</v>
       </c>
       <c r="H24" t="n">
-        <v>3217.26</v>
+        <v>2298</v>
       </c>
       <c r="I24" t="n">
-        <v>893</v>
+        <v>95</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Summer</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K24" t="b">
@@ -1591,7 +1591,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>912e85a0-2430-413c-b4f0-2c0a156cd199</t>
+          <t>c492b3e1-300b-4efa-9cf9-ff7b27184f7a</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1601,17 +1601,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ZUB-205</t>
+          <t>ZUB-669</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Industrial Dolores 76mm</t>
+          <t>Industrial Dolores 17mm</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fittings</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1620,19 +1620,15 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2454.89</v>
+        <v>3720.1</v>
       </c>
       <c r="H25" t="n">
-        <v>3050.94</v>
+        <v>5033.08</v>
       </c>
       <c r="I25" t="n">
-        <v>85</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Monsoon</t>
-        </is>
-      </c>
+        <v>686</v>
+      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="b">
         <v>0</v>
       </c>
@@ -1640,7 +1636,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9c6cae7a-f365-4ef1-b7fa-9043d257ea40</t>
+          <t>83a8185b-7aef-4810-91d8-a489885c99dc</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1650,38 +1646,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AUP-547</t>
+          <t>AUP-533</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Industrial Est 21mm</t>
+          <t>Industrial Est 16mm</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>4536</v>
+        <v>4380.68</v>
       </c>
       <c r="H26" t="n">
-        <v>5383.49</v>
+        <v>6068.48</v>
       </c>
       <c r="I26" t="n">
-        <v>905</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Summer</t>
-        </is>
-      </c>
+        <v>360</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="b">
         <v>0</v>
       </c>
@@ -1689,7 +1681,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7e6ba3df-d9ee-40f4-8317-76e2119a8644</t>
+          <t>664d2eda-e071-4e58-a888-d04c9e02cdaa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1699,46 +1691,46 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TVP-482</t>
+          <t>TVP-329</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Industrial Nostrum 40mm</t>
+          <t>Industrial Nostrum 23mm</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2132.99</v>
+        <v>1142.42</v>
       </c>
       <c r="H27" t="n">
-        <v>2664.35</v>
+        <v>1501.35</v>
       </c>
       <c r="I27" t="n">
-        <v>383</v>
+        <v>117</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Summer</t>
         </is>
       </c>
       <c r="K27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>939e63f6-4be6-4fc0-8803-1ed5303a32ad</t>
+          <t>660991be-1fa0-4dfa-a907-07aef3c5b530</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1748,32 +1740,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>RXI-765</t>
+          <t>RXI-885</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Industrial Veritatis 52mm</t>
+          <t>Industrial Veritatis 89mm</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Box</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>4661.05</v>
+        <v>4055.38</v>
       </c>
       <c r="H28" t="n">
-        <v>6338.07</v>
+        <v>5520.54</v>
       </c>
       <c r="I28" t="n">
-        <v>39</v>
+        <v>623</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1781,13 +1773,13 @@
         </is>
       </c>
       <c r="K28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6e21769d-bfe4-4273-94d5-a0326e4416c0</t>
+          <t>cfd9a9e3-f671-4150-ab02-cfd1b1e2d562</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1797,34 +1789,38 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>UVE-877</t>
+          <t>UVE-447</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Industrial Officiis 100mm</t>
+          <t>Industrial Officiis 54mm</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>2415.03</v>
+        <v>1439.02</v>
       </c>
       <c r="H29" t="n">
-        <v>3279.07</v>
+        <v>1929.15</v>
       </c>
       <c r="I29" t="n">
-        <v>630</v>
-      </c>
-      <c r="J29" t="inlineStr"/>
+        <v>890</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Monsoon</t>
+        </is>
+      </c>
       <c r="K29" t="b">
         <v>0</v>
       </c>
@@ -1832,7 +1828,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7ed541b9-6494-4258-8ebb-07c1a0ba553c</t>
+          <t>84325aff-9e1e-4629-b10d-4c21e2aa2052</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1842,36 +1838,36 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CWX-253</t>
+          <t>CWX-748</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Industrial Inventore 80mm</t>
+          <t>Industrial Inventore 13mm</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>193.12</v>
+        <v>2063.84</v>
       </c>
       <c r="H30" t="n">
-        <v>232.5</v>
+        <v>2446.62</v>
       </c>
       <c r="I30" t="n">
-        <v>113</v>
+        <v>385</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Summer</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K30" t="b">
@@ -1881,7 +1877,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>154fd94a-d274-40b7-89b0-2da39f29ffe9</t>
+          <t>6a3b4004-10d8-40bd-b945-fba820003936</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1891,17 +1887,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FJG-754</t>
+          <t>FJG-432</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Industrial Doloribus 89mm</t>
+          <t>Industrial Doloribus 82mm</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1910,19 +1906,15 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>697.0599999999999</v>
+        <v>871.3099999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>843.17</v>
+        <v>1069.89</v>
       </c>
       <c r="I31" t="n">
-        <v>113</v>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Winter</t>
-        </is>
-      </c>
+        <v>904</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
       <c r="K31" t="b">
         <v>0</v>
       </c>
@@ -1930,7 +1922,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>afba68eb-2f5a-4f6b-a9be-14df5434b064</t>
+          <t>bb8c5d15-4266-4857-9e0e-debdb76bb24b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1940,17 +1932,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PMF-347</t>
+          <t>PMF-183</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Industrial Hic 28mm</t>
+          <t>Industrial Hic 44mm</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1959,17 +1951,17 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>180.53</v>
+        <v>3796.74</v>
       </c>
       <c r="H32" t="n">
-        <v>230.87</v>
+        <v>4413.48</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>497</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Summer</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K32" t="b">
@@ -1979,7 +1971,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>c275aad5-f97a-41ba-9d42-6dba39b5ea36</t>
+          <t>181edc46-7ec7-405b-8308-f548e108cfb8</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1989,34 +1981,38 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IIM-187</t>
+          <t>IIM-453</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Industrial Fuga 77mm</t>
+          <t>Industrial Fuga 65mm</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>2141.18</v>
+        <v>1156.29</v>
       </c>
       <c r="H33" t="n">
-        <v>2817.99</v>
+        <v>1477.84</v>
       </c>
       <c r="I33" t="n">
-        <v>976</v>
-      </c>
-      <c r="J33" t="inlineStr"/>
+        <v>694</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Winter</t>
+        </is>
+      </c>
       <c r="K33" t="b">
         <v>0</v>
       </c>
@@ -2024,7 +2020,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>b32b5202-2cab-47f2-8ee5-1fd82548b626</t>
+          <t>5f1533e5-15b7-41dc-803c-1e3ba0ff852d</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2034,12 +2030,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>UOE-482</t>
+          <t>UOE-713</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Industrial Autem 42mm</t>
+          <t>Industrial Autem 17mm</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2049,19 +2045,23 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>2403.66</v>
+        <v>1611.26</v>
       </c>
       <c r="H34" t="n">
-        <v>3146.19</v>
+        <v>1941.78</v>
       </c>
       <c r="I34" t="n">
-        <v>807</v>
-      </c>
-      <c r="J34" t="inlineStr"/>
+        <v>308</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Monsoon</t>
+        </is>
+      </c>
       <c r="K34" t="b">
         <v>0</v>
       </c>
@@ -2069,7 +2069,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6024c2ed-6466-4642-9e91-71b6a1cfa46a</t>
+          <t>386d8a25-4bd5-451f-b2bd-6efe75f06d54</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2079,36 +2079,36 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BGO-890</t>
+          <t>BGO-222</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Industrial Aliquam 84mm</t>
+          <t>Industrial Aliquam 10mm</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Meters</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>3691.41</v>
+        <v>3844.39</v>
       </c>
       <c r="H35" t="n">
-        <v>4824.91</v>
+        <v>4699.24</v>
       </c>
       <c r="I35" t="n">
-        <v>45</v>
+        <v>179</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Summer</t>
+          <t>Monsoon</t>
         </is>
       </c>
       <c r="K35" t="b">
@@ -2118,7 +2118,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>33a3c8ac-3abe-484e-be37-a5c1ecbdde5a</t>
+          <t>d388e5e0-4871-41f6-abe7-d3d0be043d90</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2128,38 +2128,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LLZ-897</t>
+          <t>LLZ-953</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Industrial Rerum 97mm</t>
+          <t>Industrial Rerum 95mm</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Box</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>4086.19</v>
+        <v>3547.99</v>
       </c>
       <c r="H36" t="n">
-        <v>4877.98</v>
+        <v>4523.92</v>
       </c>
       <c r="I36" t="n">
-        <v>646</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Monsoon</t>
-        </is>
-      </c>
+        <v>406</v>
+      </c>
+      <c r="J36" t="inlineStr"/>
       <c r="K36" t="b">
         <v>0</v>
       </c>
@@ -2167,7 +2163,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>693b4889-877c-42a5-a1c6-5350d72d1809</t>
+          <t>fa3c26c0-143f-4d28-819c-0de0bdf368c2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2177,36 +2173,36 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NCJ-568</t>
+          <t>NCJ-420</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Industrial Facilis 14mm</t>
+          <t>Industrial Facilis 83mm</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Nos</t>
+          <t>Meters</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>409.19</v>
+        <v>2352.8</v>
       </c>
       <c r="H37" t="n">
-        <v>549.97</v>
+        <v>2751.52</v>
       </c>
       <c r="I37" t="n">
-        <v>44</v>
+        <v>726</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K37" t="b">
@@ -2216,7 +2212,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>a0494f20-407b-4406-8f18-de361a2f01da</t>
+          <t>5f90d643-4e75-4faf-acf5-9968d3d1d433</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2226,12 +2222,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>IIE-507</t>
+          <t>IIE-275</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Industrial Ullam 79mm</t>
+          <t>Industrial Ullam 89mm</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2245,17 +2241,17 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>1646.42</v>
+        <v>2084.66</v>
       </c>
       <c r="H38" t="n">
-        <v>2021.01</v>
+        <v>2900.91</v>
       </c>
       <c r="I38" t="n">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="K38" t="b">
@@ -2265,7 +2261,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>bf6d9392-a914-41b0-b6f7-fa005a8896f9</t>
+          <t>18199f19-daa6-46fa-aa4c-d0c4755f7bad</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2275,32 +2271,32 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>XJX-771</t>
+          <t>XJX-636</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Industrial Mollitia 52mm</t>
+          <t>Industrial Mollitia 20mm</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>4324.48</v>
+        <v>1292.25</v>
       </c>
       <c r="H39" t="n">
-        <v>5024.83</v>
+        <v>1676.33</v>
       </c>
       <c r="I39" t="n">
-        <v>818</v>
+        <v>763</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2314,7 +2310,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>aa478c04-28c8-4457-bf81-70697b22e3b6</t>
+          <t>6f116b1f-f18e-4371-b008-4f74ecb66c75</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2324,36 +2320,36 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>OXL-495</t>
+          <t>OXL-748</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Industrial Illum 53mm</t>
+          <t>Industrial Illum 24mm</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2060.11</v>
+        <v>3917.68</v>
       </c>
       <c r="H40" t="n">
-        <v>2595.6</v>
+        <v>4580.14</v>
       </c>
       <c r="I40" t="n">
-        <v>708</v>
+        <v>927</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Summer</t>
         </is>
       </c>
       <c r="K40" t="b">
@@ -2363,7 +2359,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>e40fd653-eed8-4745-a122-bc6d60c221f0</t>
+          <t>b2c2b181-4866-4303-a52a-c4140ac0941b</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2373,12 +2369,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>IDG-184</t>
+          <t>IDG-251</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Industrial Quaerat 64mm</t>
+          <t>Industrial Quaerat 40mm</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2388,17 +2384,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>4006.73</v>
+        <v>4795.29</v>
       </c>
       <c r="H41" t="n">
-        <v>4874.91</v>
+        <v>6288.36</v>
       </c>
       <c r="I41" t="n">
-        <v>616</v>
+        <v>262</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2412,7 +2408,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6762b0f8-708a-4e77-81c1-24867763abb8</t>
+          <t>e8d69c6d-834a-4735-b636-ae020a696fec</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2422,17 +2418,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FZX-776</t>
+          <t>FZX-177</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Industrial Provident 47mm</t>
+          <t>Industrial Provident 32mm</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Valves</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2441,13 +2437,13 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>1673.94</v>
+        <v>849.0599999999999</v>
       </c>
       <c r="H42" t="n">
-        <v>1958.54</v>
+        <v>1137.56</v>
       </c>
       <c r="I42" t="n">
-        <v>617</v>
+        <v>772</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2461,7 +2457,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0bc73cdb-22ab-4371-8f3d-317ab884364f</t>
+          <t>7af7a381-61a0-4649-b704-6122acab1ee1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2471,32 +2467,32 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>AQP-844</t>
+          <t>AQP-739</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Industrial Sint 55mm</t>
+          <t>Industrial Sint 51mm</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>2275.15</v>
+        <v>4422.04</v>
       </c>
       <c r="H43" t="n">
-        <v>2870.74</v>
+        <v>5796.18</v>
       </c>
       <c r="I43" t="n">
-        <v>281</v>
+        <v>450</v>
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="b">
@@ -2506,7 +2502,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0727feee-5e75-4e2a-8820-e91f165ba671</t>
+          <t>541eed14-9858-42b9-8c2c-42b9ca174785</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2516,17 +2512,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>RKW-920</t>
+          <t>RKW-705</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Industrial Quam 96mm</t>
+          <t>Industrial Quam 17mm</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2535,13 +2531,13 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>3223.81</v>
+        <v>3193.79</v>
       </c>
       <c r="H44" t="n">
-        <v>4000.19</v>
+        <v>4308.69</v>
       </c>
       <c r="I44" t="n">
-        <v>146</v>
+        <v>317</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2549,13 +2545,13 @@
         </is>
       </c>
       <c r="K44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>d69506aa-36d0-4efb-b13c-fd9ef9733d7d</t>
+          <t>1060a77b-dff2-4c01-8cf6-9cce728d70e2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2565,38 +2561,34 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ICK-475</t>
+          <t>ICK-178</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Industrial Dolorum 56mm</t>
+          <t>Industrial Dolorum 92mm</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pumps</t>
+          <t>Fittings</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Meters</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>429.44</v>
+        <v>378.76</v>
       </c>
       <c r="H45" t="n">
-        <v>577.4400000000001</v>
+        <v>514.33</v>
       </c>
       <c r="I45" t="n">
-        <v>619</v>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Monsoon</t>
-        </is>
-      </c>
+        <v>473</v>
+      </c>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="b">
         <v>0</v>
       </c>
@@ -2604,7 +2596,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>fc1e5038-a4ce-4dfc-99f3-ad770793b310</t>
+          <t>2d03f7e5-4eb6-482f-9acb-0734b519b081</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2614,17 +2606,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KKQ-881</t>
+          <t>KKQ-429</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Industrial Dignissimos 19mm</t>
+          <t>Industrial Dignissimos 87mm</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2633,19 +2625,15 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>4749.24</v>
+        <v>4068.1</v>
       </c>
       <c r="H46" t="n">
-        <v>5903.32</v>
+        <v>5341.25</v>
       </c>
       <c r="I46" t="n">
-        <v>542</v>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Summer</t>
-        </is>
-      </c>
+        <v>980</v>
+      </c>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="b">
         <v>0</v>
       </c>
@@ -2653,7 +2641,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>c57c2060-ff6f-440c-a7ce-71752cdc7e80</t>
+          <t>e71e4fa1-f4ed-454e-94f4-b23a0268405f</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2663,36 +2651,36 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>VUE-216</t>
+          <t>VUE-831</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Industrial Magnam 13mm</t>
+          <t>Industrial Magnam 20mm</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>3282.85</v>
+        <v>4073.74</v>
       </c>
       <c r="H47" t="n">
-        <v>3980.14</v>
+        <v>5537.62</v>
       </c>
       <c r="I47" t="n">
-        <v>530</v>
+        <v>40</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Monsoon</t>
         </is>
       </c>
       <c r="K47" t="b">
@@ -2702,7 +2690,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>b90dc720-4f85-497d-90db-82d21407af64</t>
+          <t>c6e59f43-de8c-49cd-9e4f-010335bb6502</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2712,17 +2700,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COW-820</t>
+          <t>COW-724</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Industrial Placeat 67mm</t>
+          <t>Industrial Placeat 30mm</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2731,17 +2719,17 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>677.03</v>
+        <v>4955.83</v>
       </c>
       <c r="H48" t="n">
-        <v>909.75</v>
+        <v>6348.5</v>
       </c>
       <c r="I48" t="n">
-        <v>710</v>
+        <v>939</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Summer</t>
         </is>
       </c>
       <c r="K48" t="b">
@@ -2751,7 +2739,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>4d9ed43d-9208-409c-891d-734b412f5200</t>
+          <t>69dc38fe-437a-4e9a-8b2b-00e85320fd9e</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2761,38 +2749,34 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>OEQ-276</t>
+          <t>OEQ-153</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Industrial Maxime 66mm</t>
+          <t>Industrial Maxime 90mm</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fittings</t>
+          <t>Valves</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Box</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>765.0700000000001</v>
+        <v>3894.88</v>
       </c>
       <c r="H49" t="n">
-        <v>893.99</v>
+        <v>5140.17</v>
       </c>
       <c r="I49" t="n">
-        <v>683</v>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Summer</t>
-        </is>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="J49" t="inlineStr"/>
       <c r="K49" t="b">
         <v>0</v>
       </c>
@@ -2800,7 +2784,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3853b733-de21-4549-904f-9f698dcce5fe</t>
+          <t>751e1bfb-bdd1-4097-a0e8-d8b22fa5f6b3</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2810,38 +2794,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>OCQ-407</t>
+          <t>OCQ-972</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Industrial Enim 30mm</t>
+          <t>Industrial Enim 94mm</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Pipes</t>
+          <t>Fasteners</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2794.99</v>
+        <v>1994.16</v>
       </c>
       <c r="H50" t="n">
-        <v>3417.13</v>
+        <v>2418.91</v>
       </c>
       <c r="I50" t="n">
-        <v>520</v>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Monsoon</t>
-        </is>
-      </c>
+        <v>341</v>
+      </c>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="b">
         <v>0</v>
       </c>
@@ -2849,7 +2829,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>bde8a8f7-9829-4219-af63-20e519047c67</t>
+          <t>629d99fd-b62f-4844-ace5-afb7e22743ad</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2859,38 +2839,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HYX-909</t>
+          <t>HYX-771</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Industrial Molestias 73mm</t>
+          <t>Industrial Molestias 99mm</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fittings</t>
+          <t>Pumps</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Nos</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1084.8</v>
+        <v>793</v>
       </c>
       <c r="H51" t="n">
-        <v>1285.18</v>
+        <v>981.3</v>
       </c>
       <c r="I51" t="n">
-        <v>567</v>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Summer</t>
-        </is>
-      </c>
+        <v>609</v>
+      </c>
+      <c r="J51" t="inlineStr"/>
       <c r="K51" t="b">
         <v>0</v>
       </c>

</xml_diff>